<commit_message>
Auto sync: Dữ liệu Giá H1 + Macro mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -1159,8 +1159,6 @@
       <c r="D38" t="n">
         <v>493.6</v>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
         <v>953.6</v>
       </c>
@@ -1170,7 +1168,6 @@
       <c r="I38" t="n">
         <v>194.8</v>
       </c>
-      <c r="J38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1183,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1630,6 +1627,26 @@
         <v>10.9</v>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>SEP 10, 2026</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>456.72</v>
+      </c>
+      <c r="C36" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>1525.481</v>
+      </c>
+      <c r="F36" t="n">
+        <v>-8.9</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1641,7 +1658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="7"/>
@@ -2541,6 +2558,48 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-14T12:00:00+0000</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>N/A (Cuối vụ)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>93% thu hoạch</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>97% đã gieo trồng</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Mỹ: 0% | Argentina: 66% (2/3 tiến độ)</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>57% Good to Excellent</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2552,7 +2611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2853,6 +2912,25 @@
       </c>
       <c r="F28" t="n">
         <v>274.66</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-11T12:00:00+0000</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>717</v>
+      </c>
+      <c r="C29" t="n">
+        <v>276.29</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1567</v>
+      </c>
+      <c r="F29" t="n">
+        <v>272.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto sync: Dữ liệu Export Sales mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1193,6 +1193,34 @@
       <c r="I39" t="n">
         <v>1683.2</v>
       </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>09/17/2026</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>267.6</v>
+      </c>
+      <c r="C40" t="n">
+        <v>-17.9</v>
+      </c>
+      <c r="D40" t="n">
+        <v>385.1</v>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>838.3</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-18.4</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1900</v>
+      </c>
+      <c r="J40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1683,7 +1711,6 @@
       <c r="C37" t="n">
         <v>-29.1</v>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>1938.523</v>
       </c>

</xml_diff>

<commit_message>
Auto sync: Dữ liệu USDA Crop Progress mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -1209,8 +1209,6 @@
       <c r="D40" t="n">
         <v>385.1</v>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
         <v>838.3</v>
       </c>
@@ -1220,7 +1218,6 @@
       <c r="I40" t="n">
         <v>1900</v>
       </c>
-      <c r="J40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1233,7 +1230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1716,6 +1713,26 @@
       </c>
       <c r="F37" t="n">
         <v>24.9</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SEP 24, 2026</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>310.635</v>
+      </c>
+      <c r="C38" t="n">
+        <v>-8.6</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>1565.924</v>
+      </c>
+      <c r="F38" t="n">
+        <v>-20.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto sync: Dữ liệu AI Điểm Tin mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1218,6 +1218,34 @@
       <c r="I40" t="n">
         <v>1900</v>
       </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>09/24/2026</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>289.3</v>
+      </c>
+      <c r="C41" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>315.4</v>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="n">
+        <v>536</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-36.1</v>
+      </c>
+      <c r="I41" t="n">
+        <v>1445.1</v>
+      </c>
+      <c r="J41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2735,7 +2763,6 @@
           <t>2026-09-28T12:00:00+0000</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -2746,7 +2773,6 @@
           <t>N/A (Cuối vụ)</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -2757,7 +2783,6 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>97% đã gieo trồng</t>

</xml_diff>

<commit_message>
Auto sync: Dữ liệu Cập nhật Phân tích & Giao diện (H1) mới
</commit_message>
<xml_diff>
--- a/USDA Reports/CBOT_Reports_History.xlsx
+++ b/USDA Reports/CBOT_Reports_History.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1293,6 +1293,34 @@
       <c r="I43" t="n">
         <v>1362.6</v>
       </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>10/15/2026</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>239.6</v>
+      </c>
+      <c r="C44" t="n">
+        <v>-25.1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>240.3</v>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="n">
+        <v>1527.1</v>
+      </c>
+      <c r="H44" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="I44" t="n">
+        <v>780.3</v>
+      </c>
+      <c r="J44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1859,7 +1887,6 @@
       <c r="C41" t="n">
         <v>-21.7</v>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
         <v>672.475</v>
       </c>

</xml_diff>